<commit_message>
add granularity to bus matrix
</commit_message>
<xml_diff>
--- a/docs/airbnb-bus-matrix.xlsx
+++ b/docs/airbnb-bus-matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git-repos\dbt-projects\dbt-airbnb-project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073B6C91-3125-4B16-9B6D-72E24B925DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FF61F9-6571-4B63-93B9-E0BDE5C89C50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{BBF274AC-B2B2-491E-9DB3-2437D80DB6CC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
   <si>
     <t>Business Process</t>
   </si>
@@ -93,6 +93,12 @@
   </si>
   <si>
     <t>Type 2</t>
+  </si>
+  <si>
+    <t>fct_listing_snapshot</t>
+  </si>
+  <si>
+    <t>Granularity</t>
   </si>
 </sst>
 </file>
@@ -500,60 +506,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79C3CDD-71DD-43A3-8B60-9119841C9FBC}">
-  <dimension ref="A2:H16"/>
+  <dimension ref="A2:I16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.81640625" customWidth="1"/>
+    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
         <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -564,77 +571,81 @@
       <c r="H3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" t="s">
-        <v>3</v>
-      </c>
       <c r="D4" t="s">
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" t="s">
         <v>4</v>
       </c>
       <c r="G4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" t="s">
         <v>3</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G14" s="5"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G15" s="5"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="D16:G16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add all snapshot files
</commit_message>
<xml_diff>
--- a/docs/airbnb-bus-matrix.xlsx
+++ b/docs/airbnb-bus-matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git-repos\dbt-projects\dbt-airbnb-project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FF61F9-6571-4B63-93B9-E0BDE5C89C50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF6C661-6520-4469-AC95-0936D48AA044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{BBF274AC-B2B2-491E-9DB3-2437D80DB6CC}"/>
   </bookViews>
@@ -533,7 +533,7 @@
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="4" t="s">

</xml_diff>

<commit_message>
docs: update busmatrix and sttm do
</commit_message>
<xml_diff>
--- a/docs/airbnb-bus-matrix.xlsx
+++ b/docs/airbnb-bus-matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git-repos\dbt-projects\dbt-airbnb-project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF6C661-6520-4469-AC95-0936D48AA044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D56979-A51D-4342-AD34-02B68B42731D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{BBF274AC-B2B2-491E-9DB3-2437D80DB6CC}"/>
   </bookViews>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
   <si>
     <t>Business Process</t>
   </si>
   <si>
-    <t>Listing Performance Snapshot</t>
-  </si>
-  <si>
     <t>Fact Table</t>
   </si>
   <si>
@@ -93,9 +90,6 @@
   </si>
   <si>
     <t>Type 2</t>
-  </si>
-  <si>
-    <t>fct_listing_snapshot</t>
   </si>
   <si>
     <t>Granularity</t>
@@ -506,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79C3CDD-71DD-43A3-8B60-9119841C9FBC}">
-  <dimension ref="A2:I16"/>
+  <dimension ref="A2:I15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.1796875" bestFit="1" customWidth="1"/>
@@ -525,95 +519,78 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" t="s">
-        <v>4</v>
-      </c>
       <c r="H3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>4</v>
-      </c>
-      <c r="G4" t="s">
-        <v>4</v>
-      </c>
-      <c r="H4" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4" t="s">
-        <v>4</v>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
+      <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="1"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="5"/>
@@ -622,7 +599,7 @@
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="5"/>
@@ -630,20 +607,11 @@
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-    </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="D13:G13"/>
     <mergeCell ref="D14:G14"/>
     <mergeCell ref="D15:G15"/>
-    <mergeCell ref="D16:G16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>